<commit_message>
Add September 27 agency confirmations and dated Brennan Cox label
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-agency-ids.xlsx
+++ b/public/records/openmhz/afpd-radio-agency-ids.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ID table" sheetId="1" r:id="Rfbc4af17c511431c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="Rb920306cfb544bd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ID table" sheetId="1" r:id="R80cb5f1f30a84254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="Rec9abc62160f4f82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -322,75 +322,97 @@
         <x:v>5J44</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
-        <x:v>2026-09-12, 2026-09-28, 2026-10-20</x:v>
+        <x:v>2026-09-12, 2026-09-27, 2026-09-28, 2026-10-20</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="2" t="str">
-        <x:v>14590038</x:v>
+        <x:v>14590031</x:v>
       </x:c>
       <x:c r="B7" s="2" t="str">
-        <x:v>5J45</x:v>
+        <x:v>5J80</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
-        <x:v>2026-09-27, 2026-10-01</x:v>
+        <x:v>2026-09-27</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:v>14590044</x:v>
+        <x:v>14590038</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
-        <x:v>5J42</x:v>
+        <x:v>5J45</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>2026-09-13, 2026-09-27, 2026-10-01, 2026-10-02</x:v>
+        <x:v>2026-09-27, 2026-10-01</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:v>14590045</x:v>
+        <x:v>14590044</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>5J51</x:v>
+        <x:v>5J42</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>2026-10-02</x:v>
+        <x:v>2026-09-13, 2026-09-27, 2026-10-01, 2026-10-02</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:v>14590237</x:v>
+        <x:v>14590045</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>5J49</x:v>
+        <x:v>5J51</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>2026-09-27</x:v>
+        <x:v>2026-10-02</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:v>14590247</x:v>
+        <x:v>14590219</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>Not supplied</x:v>
+        <x:v>5J48</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
         <x:v>2026-09-27</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="2"/>
-      <x:c r="B12" s="2"/>
-      <x:c r="C12" s="2"/>
-    </x:row>
-    <x:row r="13">
+    <x:row r="12" ht="25" customHeight="1">
+      <x:c r="A12" s="2" t="str">
+        <x:v>14590237</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="str">
+        <x:v>5J49</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="2" t="str">
+        <x:v>14590247</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="str">
+        <x:v>Not supplied</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2"/>
+      <x:c r="B14" s="2"/>
+      <x:c r="C14" s="2"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2" t="str">
         <x:v>Confirmations apply to the listed dates. See Evidence for the listening source.</x:v>
       </x:c>
-      <x:c r="B13" s="2"/>
-      <x:c r="C13" s="2"/>
+      <x:c r="B15" s="2"/>
+      <x:c r="C15" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -703,23 +725,83 @@
         <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="2"/>
-      <x:c r="B18" s="2"/>
-      <x:c r="C18" s="2"/>
-      <x:c r="D18" s="2"/>
-      <x:c r="E18" s="2"/>
-      <x:c r="F18" s="2"/>
-    </x:row>
-    <x:row r="19">
+    <x:row r="18" ht="25" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>14590219</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>5J48</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="d">
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="2" t="str">
+        <x:v>14590031</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>5J80</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="d">
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="25" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>14580155</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>5J44</x:v>
+      </x:c>
+      <x:c r="C20" s="6" t="d">
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2"/>
+      <x:c r="B21" s="2"/>
+      <x:c r="C21" s="2"/>
+      <x:c r="D21" s="2"/>
+      <x:c r="E21" s="2"/>
+      <x:c r="F21" s="2"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="str">
         <x:v>Dates are dates heard; exact clip timestamps were not supplied.</x:v>
       </x:c>
-      <x:c r="B19" s="2"/>
-      <x:c r="C19" s="2"/>
-      <x:c r="D19" s="2"/>
-      <x:c r="E19" s="2"/>
-      <x:c r="F19" s="2"/>
+      <x:c r="B22" s="2"/>
+      <x:c r="C22" s="2"/>
+      <x:c r="D22" s="2"/>
+      <x:c r="E22" s="2"/>
+      <x:c r="F22" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Carry strong radio associations to Law 2-only dates and add September 27 ID evidence
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-agency-ids.xlsx
+++ b/public/records/openmhz/afpd-radio-agency-ids.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ID table" sheetId="1" r:id="R80cb5f1f30a84254"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="Rec9abc62160f4f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ID table" sheetId="1" r:id="R2bb8b26e5df8410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="Racb78b33c4b64a5d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -366,15 +366,15 @@
         <x:v>5J51</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>2026-10-02</x:v>
+        <x:v>2026-09-27, 2026-10-02</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:v>14590219</x:v>
+        <x:v>14590072</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>5J48</x:v>
+        <x:v>5J29</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
         <x:v>2026-09-27</x:v>
@@ -382,10 +382,10 @@
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="2" t="str">
-        <x:v>14590237</x:v>
+        <x:v>14590219</x:v>
       </x:c>
       <x:c r="B12" s="2" t="str">
-        <x:v>5J49</x:v>
+        <x:v>5J48</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
         <x:v>2026-09-27</x:v>
@@ -393,26 +393,37 @@
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>14590247</x:v>
+        <x:v>14590237</x:v>
       </x:c>
       <x:c r="B13" s="2" t="str">
-        <x:v>Not supplied</x:v>
+        <x:v>5J49</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
         <x:v>2026-09-27</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="2"/>
-      <x:c r="B14" s="2"/>
-      <x:c r="C14" s="2"/>
+    <x:row r="14" ht="25" customHeight="1">
+      <x:c r="A14" s="2" t="str">
+        <x:v>14590247</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="str">
+        <x:v>Not supplied</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>2026-09-27</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="2" t="str">
-        <x:v>Confirmations apply to the listed dates. See Evidence for the listening source.</x:v>
-      </x:c>
+      <x:c r="A15" s="2"/>
       <x:c r="B15" s="2"/>
       <x:c r="C15" s="2"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="str">
+        <x:v>Confirmations apply to the listed dates. See Evidence for the listening source.</x:v>
+      </x:c>
+      <x:c r="B16" s="2"/>
+      <x:c r="C16" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -785,23 +796,63 @@
         <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-      <x:c r="D21" s="2"/>
-      <x:c r="E21" s="2"/>
-      <x:c r="F21" s="2"/>
-    </x:row>
-    <x:row r="22">
+    <x:row r="21" ht="25" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>14590072</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>5J29</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="d">
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="2" t="str">
+        <x:v>14590045</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>5J51</x:v>
+      </x:c>
+      <x:c r="C22" s="6" t="d">
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F22" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2"/>
+      <x:c r="B23" s="2"/>
+      <x:c r="C23" s="2"/>
+      <x:c r="D23" s="2"/>
+      <x:c r="E23" s="2"/>
+      <x:c r="F23" s="2"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2" t="str">
         <x:v>Dates are dates heard; exact clip timestamps were not supplied.</x:v>
       </x:c>
-      <x:c r="B22" s="2"/>
-      <x:c r="C22" s="2"/>
-      <x:c r="D22" s="2"/>
-      <x:c r="E22" s="2"/>
-      <x:c r="F22" s="2"/>
+      <x:c r="B24" s="2"/>
+      <x:c r="C24" s="2"/>
+      <x:c r="D24" s="2"/>
+      <x:c r="E24" s="2"/>
+      <x:c r="F24" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update Law 2 ID evidence for September 27, 29 and 30 in page and downloads
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-agency-ids.xlsx
+++ b/public/records/openmhz/afpd-radio-agency-ids.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ID table" sheetId="1" r:id="R2bb8b26e5df8410e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="Racb78b33c4b64a5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ID table" sheetId="1" r:id="R120c251109e3445d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="R43968e1d9f4845ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -311,7 +311,7 @@
         <x:v>5J53</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>Not supplied</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
@@ -327,76 +327,76 @@
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="2" t="str">
-        <x:v>14590031</x:v>
+        <x:v>14590021</x:v>
       </x:c>
       <x:c r="B7" s="2" t="str">
-        <x:v>5J80</x:v>
+        <x:v>5J46</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
-        <x:v>2026-09-27</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:v>14590038</x:v>
+        <x:v>14590030</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
-        <x:v>5J45</x:v>
+        <x:v>5J36</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>2026-09-27, 2026-10-01</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:v>14590044</x:v>
+        <x:v>14590031</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>5J42</x:v>
+        <x:v>5J80</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>2026-09-13, 2026-09-27, 2026-10-01, 2026-10-02</x:v>
+        <x:v>2026-09-27</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:v>14590045</x:v>
+        <x:v>14590038</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>5J51</x:v>
+        <x:v>5J45</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>2026-09-27, 2026-10-02</x:v>
+        <x:v>2026-09-27, 2026-10-01</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:v>14590072</x:v>
+        <x:v>14590044</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>5J29</x:v>
+        <x:v>5J42</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
-        <x:v>2026-09-27</x:v>
+        <x:v>2026-09-13, 2026-09-27, 2026-10-01, 2026-10-02</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="2" t="str">
-        <x:v>14590219</x:v>
+        <x:v>14590045</x:v>
       </x:c>
       <x:c r="B12" s="2" t="str">
-        <x:v>5J48</x:v>
+        <x:v>5J51</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
-        <x:v>2026-09-27</x:v>
+        <x:v>2026-09-27, 2026-10-02</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>14590237</x:v>
+        <x:v>14590072</x:v>
       </x:c>
       <x:c r="B13" s="2" t="str">
-        <x:v>5J49</x:v>
+        <x:v>5J29</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
         <x:v>2026-09-27</x:v>
@@ -404,26 +404,92 @@
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="2" t="str">
+        <x:v>14590111</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="str">
+        <x:v>5J6</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="25" customHeight="1">
+      <x:c r="A15" s="2" t="str">
+        <x:v>14590206</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="str">
+        <x:v>5J50</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="25" customHeight="1">
+      <x:c r="A16" s="2" t="str">
+        <x:v>14590219</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="str">
+        <x:v>5J48</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="25" customHeight="1">
+      <x:c r="A17" s="2" t="str">
+        <x:v>14590221</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="str">
+        <x:v>5J29</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="25" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>14590237</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>5J49</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="25" customHeight="1">
+      <x:c r="A19" s="2" t="str">
         <x:v>14590247</x:v>
       </x:c>
-      <x:c r="B14" s="2" t="str">
-        <x:v>Not supplied</x:v>
-      </x:c>
-      <x:c r="C14" s="2" t="str">
-        <x:v>2026-09-27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="2"/>
-      <x:c r="C15" s="2"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="2" t="str">
+      <x:c r="B19" s="2" t="str">
+        <x:v>5J52</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>2026-09-27, 2026-09-30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="25" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>14590268</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>5J43</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2"/>
+      <x:c r="B21" s="2"/>
+      <x:c r="C21" s="2"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="str">
         <x:v>Confirmations apply to the listed dates. See Evidence for the listening source.</x:v>
       </x:c>
-      <x:c r="B16" s="2"/>
-      <x:c r="C16" s="2"/>
+      <x:c r="B22" s="2"/>
+      <x:c r="C22" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -482,19 +548,23 @@
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>14580151</x:v>
+        <x:v>14580155</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>5J53</x:v>
-      </x:c>
-      <x:c r="C5" s="6"/>
+        <x:v>5J44</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="d">
+        <x:v>2026-09-12T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="D5" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
       </x:c>
       <x:c r="E5" s="2" t="str">
-        <x:v>Owner confirmation; date not supplied</x:v>
-      </x:c>
-      <x:c r="F5" s="2" t="str"/>
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-12</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="2" t="str">
@@ -504,7 +574,7 @@
         <x:v>5J44</x:v>
       </x:c>
       <x:c r="C6" s="6" t="d">
-        <x:v>2026-09-12T00:00:00.000Z</x:v>
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -513,7 +583,7 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F6" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-12</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-28</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
@@ -524,7 +594,7 @@
         <x:v>5J44</x:v>
       </x:c>
       <x:c r="C7" s="6" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D7" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -533,18 +603,18 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F7" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-28</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-10-20</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:v>14580155</x:v>
+        <x:v>14590038</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
-        <x:v>5J44</x:v>
+        <x:v>5J45</x:v>
       </x:c>
       <x:c r="C8" s="6" t="d">
-        <x:v>2026-10-20T00:00:00.000Z</x:v>
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -553,7 +623,7 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F8" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-10-20</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
@@ -564,7 +634,7 @@
         <x:v>5J45</x:v>
       </x:c>
       <x:c r="C9" s="6" t="d">
-        <x:v>2026-09-27T00:00:00.000Z</x:v>
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -573,18 +643,18 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F9" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-10-01</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:v>14590038</x:v>
+        <x:v>14590044</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>5J45</x:v>
+        <x:v>5J42</x:v>
       </x:c>
       <x:c r="C10" s="6" t="d">
-        <x:v>2026-10-01T00:00:00.000Z</x:v>
+        <x:v>2026-09-13T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D10" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -593,7 +663,7 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F10" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-10-01</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-13</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
@@ -604,7 +674,7 @@
         <x:v>5J42</x:v>
       </x:c>
       <x:c r="C11" s="6" t="d">
-        <x:v>2026-09-13T00:00:00.000Z</x:v>
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D11" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -613,7 +683,7 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F11" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-13</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
@@ -624,7 +694,7 @@
         <x:v>5J42</x:v>
       </x:c>
       <x:c r="C12" s="6" t="d">
-        <x:v>2026-09-27T00:00:00.000Z</x:v>
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D12" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -633,7 +703,7 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F12" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-10-01</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
@@ -644,7 +714,7 @@
         <x:v>5J42</x:v>
       </x:c>
       <x:c r="C13" s="6" t="d">
-        <x:v>2026-10-01T00:00:00.000Z</x:v>
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D13" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -653,15 +723,15 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F13" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-10-01</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-10-02</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>14590044</x:v>
+        <x:v>14590045</x:v>
       </x:c>
       <x:c r="B14" s="2" t="str">
-        <x:v>5J42</x:v>
+        <x:v>5J51</x:v>
       </x:c>
       <x:c r="C14" s="6" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -678,13 +748,13 @@
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="2" t="str">
-        <x:v>14590045</x:v>
+        <x:v>14590237</x:v>
       </x:c>
       <x:c r="B15" s="2" t="str">
-        <x:v>5J51</x:v>
+        <x:v>5J49</x:v>
       </x:c>
       <x:c r="C15" s="6" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D15" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -693,15 +763,15 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F15" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-10-02</x:v>
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="2" t="str">
-        <x:v>14590237</x:v>
+        <x:v>14590247</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>5J49</x:v>
+        <x:v>5J52</x:v>
       </x:c>
       <x:c r="C16" s="6" t="d">
         <x:v>2026-09-27T00:00:00.000Z</x:v>
@@ -718,10 +788,10 @@
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="2" t="str">
-        <x:v>14590247</x:v>
+        <x:v>14590219</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>Not supplied</x:v>
+        <x:v>5J48</x:v>
       </x:c>
       <x:c r="C17" s="6" t="d">
         <x:v>2026-09-27T00:00:00.000Z</x:v>
@@ -730,7 +800,7 @@
         <x:v>Law 2 (5922)</x:v>
       </x:c>
       <x:c r="E17" s="2" t="str">
-        <x:v>Owner supplied date; 5J identifier not supplied</x:v>
+        <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F17" s="2" t="str">
         <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
@@ -738,10 +808,10 @@
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>14590219</x:v>
+        <x:v>14590031</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>5J48</x:v>
+        <x:v>5J80</x:v>
       </x:c>
       <x:c r="C18" s="6" t="d">
         <x:v>2026-09-27T00:00:00.000Z</x:v>
@@ -758,10 +828,10 @@
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="2" t="str">
-        <x:v>14590031</x:v>
+        <x:v>14580155</x:v>
       </x:c>
       <x:c r="B19" s="2" t="str">
-        <x:v>5J80</x:v>
+        <x:v>5J44</x:v>
       </x:c>
       <x:c r="C19" s="6" t="d">
         <x:v>2026-09-27T00:00:00.000Z</x:v>
@@ -778,10 +848,10 @@
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="2" t="str">
-        <x:v>14580155</x:v>
+        <x:v>14590072</x:v>
       </x:c>
       <x:c r="B20" s="2" t="str">
-        <x:v>5J44</x:v>
+        <x:v>5J29</x:v>
       </x:c>
       <x:c r="C20" s="6" t="d">
         <x:v>2026-09-27T00:00:00.000Z</x:v>
@@ -798,10 +868,10 @@
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="2" t="str">
-        <x:v>14590072</x:v>
+        <x:v>14590045</x:v>
       </x:c>
       <x:c r="B21" s="2" t="str">
-        <x:v>5J29</x:v>
+        <x:v>5J51</x:v>
       </x:c>
       <x:c r="C21" s="6" t="d">
         <x:v>2026-09-27T00:00:00.000Z</x:v>
@@ -818,13 +888,13 @@
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="2" t="str">
-        <x:v>14590045</x:v>
+        <x:v>14590030</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>5J51</x:v>
+        <x:v>5J36</x:v>
       </x:c>
       <x:c r="C22" s="6" t="d">
-        <x:v>2026-09-27T00:00:00.000Z</x:v>
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D22" s="2" t="str">
         <x:v>Law 2 (5922)</x:v>
@@ -833,26 +903,166 @@
         <x:v>Owner listening confirmation</x:v>
       </x:c>
       <x:c r="F22" s="2" t="str">
-        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="2"/>
-      <x:c r="B23" s="2"/>
-      <x:c r="C23" s="2"/>
-      <x:c r="D23" s="2"/>
-      <x:c r="E23" s="2"/>
-      <x:c r="F23" s="2"/>
-    </x:row>
-    <x:row r="24">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="25" customHeight="1">
+      <x:c r="A23" s="2" t="str">
+        <x:v>14590021</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>5J46</x:v>
+      </x:c>
+      <x:c r="C23" s="6" t="d">
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F23" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="25" customHeight="1">
       <x:c r="A24" s="2" t="str">
+        <x:v>14590206</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="str">
+        <x:v>5J50</x:v>
+      </x:c>
+      <x:c r="C24" s="6" t="d">
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D24" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F24" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="25" customHeight="1">
+      <x:c r="A25" s="2" t="str">
+        <x:v>14590268</x:v>
+      </x:c>
+      <x:c r="B25" s="2" t="str">
+        <x:v>5J43</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="d">
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F25" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="25" customHeight="1">
+      <x:c r="A26" s="2" t="str">
+        <x:v>14580151</x:v>
+      </x:c>
+      <x:c r="B26" s="2" t="str">
+        <x:v>5J53</x:v>
+      </x:c>
+      <x:c r="C26" s="6" t="d">
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D26" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E26" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F26" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="25" customHeight="1">
+      <x:c r="A27" s="2" t="str">
+        <x:v>14590221</x:v>
+      </x:c>
+      <x:c r="B27" s="2" t="str">
+        <x:v>5J29</x:v>
+      </x:c>
+      <x:c r="C27" s="6" t="d">
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F27" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="25" customHeight="1">
+      <x:c r="A28" s="2" t="str">
+        <x:v>14590247</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="str">
+        <x:v>5J52</x:v>
+      </x:c>
+      <x:c r="C28" s="6" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F28" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="25" customHeight="1">
+      <x:c r="A29" s="2" t="str">
+        <x:v>14590111</x:v>
+      </x:c>
+      <x:c r="B29" s="2" t="str">
+        <x:v>5J6</x:v>
+      </x:c>
+      <x:c r="C29" s="6" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F29" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="2"/>
+      <x:c r="B30" s="2"/>
+      <x:c r="C30" s="2"/>
+      <x:c r="D30" s="2"/>
+      <x:c r="E30" s="2"/>
+      <x:c r="F30" s="2"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2" t="str">
         <x:v>Dates are dates heard; exact clip timestamps were not supplied.</x:v>
       </x:c>
-      <x:c r="B24" s="2"/>
-      <x:c r="C24" s="2"/>
-      <x:c r="D24" s="2"/>
-      <x:c r="E24" s="2"/>
-      <x:c r="F24" s="2"/>
+      <x:c r="B31" s="2"/>
+      <x:c r="C31" s="2"/>
+      <x:c r="D31" s="2"/>
+      <x:c r="E31" s="2"/>
+      <x:c r="F31" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update September 27 IDs-only 5J6 CSV and workbook
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-agency-ids.xlsx
+++ b/public/records/openmhz/afpd-radio-agency-ids.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ID table" sheetId="1" r:id="R120c251109e3445d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="R43968e1d9f4845ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ID table" sheetId="1" r:id="R9510ba093abb44a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="R72c51a95162849ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,92 +404,103 @@
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>14590111</x:v>
+        <x:v>14590089</x:v>
       </x:c>
       <x:c r="B14" s="2" t="str">
         <x:v>5J6</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
-        <x:v>2026-09-30</x:v>
+        <x:v>2026-09-27</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="2" t="str">
-        <x:v>14590206</x:v>
+        <x:v>14590111</x:v>
       </x:c>
       <x:c r="B15" s="2" t="str">
-        <x:v>5J50</x:v>
+        <x:v>5J6</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-27, 2026-09-30</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="2" t="str">
-        <x:v>14590219</x:v>
+        <x:v>14590206</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>5J48</x:v>
+        <x:v>5J50</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
-        <x:v>2026-09-27</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="2" t="str">
-        <x:v>14590221</x:v>
+        <x:v>14590219</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>5J29</x:v>
+        <x:v>5J48</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-27</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>14590237</x:v>
+        <x:v>14590221</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>5J49</x:v>
+        <x:v>5J29</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
-        <x:v>2026-09-27</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="2" t="str">
-        <x:v>14590247</x:v>
+        <x:v>14590237</x:v>
       </x:c>
       <x:c r="B19" s="2" t="str">
-        <x:v>5J52</x:v>
+        <x:v>5J49</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
-        <x:v>2026-09-27, 2026-09-30</x:v>
+        <x:v>2026-09-27</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="2" t="str">
+        <x:v>14590247</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>5J52</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>2026-09-27, 2026-09-30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="25" customHeight="1">
+      <x:c r="A21" s="2" t="str">
         <x:v>14590268</x:v>
       </x:c>
-      <x:c r="B20" s="2" t="str">
+      <x:c r="B21" s="2" t="str">
         <x:v>5J43</x:v>
       </x:c>
-      <x:c r="C20" s="2" t="str">
+      <x:c r="C21" s="2" t="str">
         <x:v>2026-09-29</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-    </x:row>
     <x:row r="22">
-      <x:c r="A22" s="2" t="str">
-        <x:v>Confirmations apply to the listed dates. See Evidence for the listening source.</x:v>
-      </x:c>
+      <x:c r="A22" s="2"/>
       <x:c r="B22" s="2"/>
       <x:c r="C22" s="2"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="str">
+        <x:v>Confirmations apply to the listed dates. See Evidence for the listening source.</x:v>
+      </x:c>
+      <x:c r="B23" s="2"/>
+      <x:c r="C23" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1046,23 +1057,63 @@
         <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-30</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="2"/>
-      <x:c r="B30" s="2"/>
-      <x:c r="C30" s="2"/>
-      <x:c r="D30" s="2"/>
-      <x:c r="E30" s="2"/>
-      <x:c r="F30" s="2"/>
-    </x:row>
-    <x:row r="31">
+    <x:row r="30" ht="25" customHeight="1">
+      <x:c r="A30" s="2" t="str">
+        <x:v>14590089</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>5J6</x:v>
+      </x:c>
+      <x:c r="C30" s="6" t="d">
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F30" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="25" customHeight="1">
       <x:c r="A31" s="2" t="str">
+        <x:v>14590111</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>5J6</x:v>
+      </x:c>
+      <x:c r="C31" s="6" t="d">
+        <x:v>2026-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>Law 2 (5922)</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str">
+        <x:v>Owner listening confirmation</x:v>
+      </x:c>
+      <x:c r="F31" s="2" t="str">
+        <x:v>https://afpd-accountability.com/law-2-radio/?date=2026-09-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2"/>
+      <x:c r="B32" s="2"/>
+      <x:c r="C32" s="2"/>
+      <x:c r="D32" s="2"/>
+      <x:c r="E32" s="2"/>
+      <x:c r="F32" s="2"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="2" t="str">
         <x:v>Dates are dates heard; exact clip timestamps were not supplied.</x:v>
       </x:c>
-      <x:c r="B31" s="2"/>
-      <x:c r="C31" s="2"/>
-      <x:c r="D31" s="2"/>
-      <x:c r="E31" s="2"/>
-      <x:c r="F31" s="2"/>
+      <x:c r="B33" s="2"/>
+      <x:c r="C33" s="2"/>
+      <x:c r="D33" s="2"/>
+      <x:c r="E33" s="2"/>
+      <x:c r="F33" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>